<commit_message>
refactor(parser): build AST directly with semantic value stack
</commit_message>
<xml_diff>
--- a/实验设计/语法分析/语法表格/文法表.xlsx
+++ b/实验设计/语法分析/语法表格/文法表.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文法产生式" sheetId="1" r:id="R2fd1261f1f994a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文法产生式" sheetId="1" r:id="R9ea5f0e48a694ca8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -454,7 +454,7 @@
         <x:v>run</x:v>
       </x:c>
       <x:c r="E8" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:391</x:v>
+        <x:v>src/语法分析/parser.cpp:313</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
@@ -471,7 +471,7 @@
         <x:v>run</x:v>
       </x:c>
       <x:c r="E9" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:391</x:v>
+        <x:v>src/语法分析/parser.cpp:313</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
@@ -488,7 +488,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E10" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
@@ -505,7 +505,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E11" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -522,7 +522,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E12" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
@@ -539,7 +539,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E13" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
@@ -556,7 +556,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E14" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
@@ -573,7 +573,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E15" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
@@ -590,7 +590,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E16" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
@@ -607,7 +607,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E17" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -624,7 +624,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E18" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
@@ -641,7 +641,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E19" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
@@ -658,7 +658,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E20" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
@@ -675,7 +675,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E21" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
@@ -692,7 +692,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E22" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
@@ -709,7 +709,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E23" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
@@ -726,7 +726,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E24" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
@@ -743,7 +743,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E25" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
@@ -760,7 +760,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E26" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
@@ -777,7 +777,7 @@
         <x:v>specs</x:v>
       </x:c>
       <x:c r="E27" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:82</x:v>
+        <x:v>src/语法分析/parser.cpp:81</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
@@ -794,7 +794,7 @@
         <x:v>specs</x:v>
       </x:c>
       <x:c r="E28" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:82</x:v>
+        <x:v>src/语法分析/parser.cpp:81</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
@@ -811,7 +811,7 @@
         <x:v>specs</x:v>
       </x:c>
       <x:c r="E29" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:82</x:v>
+        <x:v>src/语法分析/parser.cpp:81</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
@@ -828,7 +828,7 @@
         <x:v>specs</x:v>
       </x:c>
       <x:c r="E30" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:82</x:v>
+        <x:v>src/语法分析/parser.cpp:81</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
@@ -845,7 +845,7 @@
         <x:v>specs</x:v>
       </x:c>
       <x:c r="E31" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:82</x:v>
+        <x:v>src/语法分析/parser.cpp:81</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
@@ -862,7 +862,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E32" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
@@ -879,7 +879,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E33" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="24" customHeight="1">
@@ -896,7 +896,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E34" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
@@ -913,7 +913,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E35" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="24" customHeight="1">
@@ -930,7 +930,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E36" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:133</x:v>
+        <x:v>src/语法分析/parser.cpp:122</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="24" customHeight="1">
@@ -947,7 +947,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E37" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:94</x:v>
+        <x:v>src/语法分析/parser.cpp:93</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="24" customHeight="1">
@@ -964,7 +964,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E38" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:94</x:v>
+        <x:v>src/语法分析/parser.cpp:93</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="24" customHeight="1">
@@ -981,7 +981,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E39" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:94</x:v>
+        <x:v>src/语法分析/parser.cpp:93</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="24" customHeight="1">
@@ -998,7 +998,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E40" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:94</x:v>
+        <x:v>src/语法分析/parser.cpp:93</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="24" customHeight="1">
@@ -1015,7 +1015,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E41" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:94</x:v>
+        <x:v>src/语法分析/parser.cpp:93</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="24" customHeight="1">
@@ -1032,7 +1032,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E42" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:94</x:v>
+        <x:v>src/语法分析/parser.cpp:93</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="24" customHeight="1">
@@ -1049,7 +1049,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E43" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:94</x:v>
+        <x:v>src/语法分析/parser.cpp:93</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="24" customHeight="1">
@@ -1066,7 +1066,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E44" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:94</x:v>
+        <x:v>src/语法分析/parser.cpp:93</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="24" customHeight="1">
@@ -1083,7 +1083,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E45" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:94</x:v>
+        <x:v>src/语法分析/parser.cpp:93</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="24" customHeight="1">
@@ -1100,7 +1100,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E46" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:94</x:v>
+        <x:v>src/语法分析/parser.cpp:93</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="24" customHeight="1">
@@ -1117,7 +1117,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E47" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:94</x:v>
+        <x:v>src/语法分析/parser.cpp:93</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="24" customHeight="1">
@@ -1134,7 +1134,7 @@
         <x:v>block</x:v>
       </x:c>
       <x:c r="E48" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:188</x:v>
+        <x:v>src/语法分析/parser.cpp:147</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="24" customHeight="1">
@@ -1151,7 +1151,7 @@
         <x:v>block</x:v>
       </x:c>
       <x:c r="E49" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:188</x:v>
+        <x:v>src/语法分析/parser.cpp:147</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="24" customHeight="1">
@@ -1168,7 +1168,7 @@
         <x:v>block</x:v>
       </x:c>
       <x:c r="E50" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:188</x:v>
+        <x:v>src/语法分析/parser.cpp:147</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="24" customHeight="1">
@@ -1185,7 +1185,7 @@
         <x:v>block</x:v>
       </x:c>
       <x:c r="E51" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:188</x:v>
+        <x:v>src/语法分析/parser.cpp:147</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="24" customHeight="1">
@@ -1202,7 +1202,7 @@
         <x:v>block</x:v>
       </x:c>
       <x:c r="E52" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:188</x:v>
+        <x:v>src/语法分析/parser.cpp:147</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="24" customHeight="1">
@@ -1219,7 +1219,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E53" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:203</x:v>
+        <x:v>src/语法分析/parser.cpp:153</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="24" customHeight="1">
@@ -1236,7 +1236,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E54" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:203</x:v>
+        <x:v>src/语法分析/parser.cpp:153</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="24" customHeight="1">
@@ -1253,7 +1253,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E55" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:203</x:v>
+        <x:v>src/语法分析/parser.cpp:153</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="24" customHeight="1">
@@ -1270,7 +1270,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E56" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:203</x:v>
+        <x:v>src/语法分析/parser.cpp:153</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="24" customHeight="1">
@@ -1287,7 +1287,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E57" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:203</x:v>
+        <x:v>src/语法分析/parser.cpp:153</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="24" customHeight="1">
@@ -1304,7 +1304,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E58" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:203</x:v>
+        <x:v>src/语法分析/parser.cpp:153</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="24" customHeight="1">
@@ -1321,7 +1321,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E59" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:203</x:v>
+        <x:v>src/语法分析/parser.cpp:153</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="24" customHeight="1">
@@ -1338,7 +1338,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E60" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:203</x:v>
+        <x:v>src/语法分析/parser.cpp:153</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="24" customHeight="1">
@@ -1355,7 +1355,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E61" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:203</x:v>
+        <x:v>src/语法分析/parser.cpp:153</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="24" customHeight="1">
@@ -1372,7 +1372,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E62" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:203</x:v>
+        <x:v>src/语法分析/parser.cpp:153</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="24" customHeight="1">
@@ -1389,7 +1389,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E63" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:203</x:v>
+        <x:v>src/语法分析/parser.cpp:153</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="24" customHeight="1">
@@ -1406,7 +1406,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E64" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:203</x:v>
+        <x:v>src/语法分析/parser.cpp:153</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="24" customHeight="1">
@@ -1423,7 +1423,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E65" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:203</x:v>
+        <x:v>src/语法分析/parser.cpp:153</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="24" customHeight="1">
@@ -1440,7 +1440,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E66" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="24" customHeight="1">
@@ -1457,7 +1457,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E67" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="24" customHeight="1">
@@ -1474,7 +1474,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E68" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="24" customHeight="1">
@@ -1491,7 +1491,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E69" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="24" customHeight="1">
@@ -1508,7 +1508,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E70" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="24" customHeight="1">
@@ -1525,7 +1525,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E71" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="24" customHeight="1">
@@ -1542,7 +1542,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E72" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="24" customHeight="1">
@@ -1559,7 +1559,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E73" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="24" customHeight="1">
@@ -1576,7 +1576,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E74" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="24" customHeight="1">
@@ -1593,7 +1593,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E75" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="24" customHeight="1">
@@ -1610,7 +1610,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E76" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="24" customHeight="1">
@@ -1627,7 +1627,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E77" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="24" customHeight="1">
@@ -1644,7 +1644,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E78" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="24" customHeight="1">
@@ -1661,7 +1661,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E79" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="24" customHeight="1">
@@ -1678,7 +1678,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E80" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="24" customHeight="1">
@@ -1695,7 +1695,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E81" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="24" customHeight="1">
@@ -1712,7 +1712,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E82" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="24" customHeight="1">
@@ -1729,7 +1729,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E83" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="24" customHeight="1">
@@ -1746,7 +1746,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E84" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="24" customHeight="1">
@@ -1763,7 +1763,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E85" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="24" customHeight="1">
@@ -1780,7 +1780,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E86" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="24" customHeight="1">
@@ -1797,7 +1797,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E87" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="24" customHeight="1">
@@ -1814,7 +1814,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E88" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="24" customHeight="1">
@@ -1831,7 +1831,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E89" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="24" customHeight="1">
@@ -1848,7 +1848,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E90" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="24" customHeight="1">
@@ -1865,7 +1865,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E91" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="24" customHeight="1">
@@ -1882,7 +1882,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E92" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="24" customHeight="1">
@@ -1899,7 +1899,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E93" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:233</x:v>
+        <x:v>src/语法分析/parser.cpp:179</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="24" customHeight="1">
@@ -1916,7 +1916,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E94" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="24" customHeight="1">
@@ -1933,7 +1933,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E95" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="24" customHeight="1">
@@ -1950,7 +1950,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E96" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="24" customHeight="1">
@@ -1967,7 +1967,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E97" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="24" customHeight="1">
@@ -1984,7 +1984,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E98" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="24" customHeight="1">
@@ -2001,7 +2001,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E99" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="24" customHeight="1">
@@ -2018,7 +2018,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E100" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="24" customHeight="1">
@@ -2035,7 +2035,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E101" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="24" customHeight="1">
@@ -2052,7 +2052,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E102" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="24" customHeight="1">
@@ -2069,7 +2069,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E103" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="24" customHeight="1">
@@ -2086,7 +2086,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E104" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="24" customHeight="1">
@@ -2103,7 +2103,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E105" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="24" customHeight="1">
@@ -2120,7 +2120,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E106" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="24" customHeight="1">
@@ -2137,7 +2137,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E107" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="24" customHeight="1">
@@ -2154,7 +2154,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E108" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:256</x:v>
+        <x:v>src/语法分析/parser.cpp:190</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="24" customHeight="1">
@@ -2171,7 +2171,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E109" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:292</x:v>
+        <x:v>src/语法分析/parser.cpp:217</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="24" customHeight="1">
@@ -2188,7 +2188,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E110" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:292</x:v>
+        <x:v>src/语法分析/parser.cpp:217</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="24" customHeight="1">
@@ -2205,7 +2205,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E111" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:292</x:v>
+        <x:v>src/语法分析/parser.cpp:217</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="24" customHeight="1">
@@ -2222,7 +2222,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E112" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:292</x:v>
+        <x:v>src/语法分析/parser.cpp:217</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="24" customHeight="1">
@@ -2239,7 +2239,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E113" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:292</x:v>
+        <x:v>src/语法分析/parser.cpp:217</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="24" customHeight="1">
@@ -2256,7 +2256,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E114" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:292</x:v>
+        <x:v>src/语法分析/parser.cpp:217</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="24" customHeight="1">
@@ -2273,7 +2273,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E115" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:292</x:v>
+        <x:v>src/语法分析/parser.cpp:217</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="24" customHeight="1">
@@ -2290,7 +2290,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E116" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:292</x:v>
+        <x:v>src/语法分析/parser.cpp:217</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="24" customHeight="1">
@@ -2307,7 +2307,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E117" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:292</x:v>
+        <x:v>src/语法分析/parser.cpp:217</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2318,7 +2318,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4daa5cfc8434297"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde842d4fbcc04a0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
refactor(parser): stop at the first syntax error
</commit_message>
<xml_diff>
--- a/实验设计/语法分析/语法表格/文法表.xlsx
+++ b/实验设计/语法分析/语法表格/文法表.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文法产生式" sheetId="1" r:id="R9ea5f0e48a694ca8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文法产生式" sheetId="1" r:id="Ra04baa607d604d79"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -454,7 +454,7 @@
         <x:v>run</x:v>
       </x:c>
       <x:c r="E8" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:313</x:v>
+        <x:v>src/语法分析/parser.cpp:289</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
@@ -471,7 +471,7 @@
         <x:v>run</x:v>
       </x:c>
       <x:c r="E9" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:313</x:v>
+        <x:v>src/语法分析/parser.cpp:289</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
@@ -488,7 +488,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E10" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
@@ -505,7 +505,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E11" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -522,7 +522,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E12" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
@@ -539,7 +539,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E13" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
@@ -556,7 +556,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E14" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
@@ -573,7 +573,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E15" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
@@ -590,7 +590,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E16" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
@@ -607,7 +607,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E17" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -624,7 +624,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E18" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
@@ -641,7 +641,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E19" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
@@ -658,7 +658,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E20" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
@@ -675,7 +675,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E21" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
@@ -692,7 +692,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E22" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
@@ -709,7 +709,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E23" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
@@ -726,7 +726,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E24" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
@@ -743,7 +743,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E25" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
@@ -760,7 +760,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E26" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
@@ -777,7 +777,7 @@
         <x:v>specs</x:v>
       </x:c>
       <x:c r="E27" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:81</x:v>
+        <x:v>src/语法分析/parser.cpp:71</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
@@ -794,7 +794,7 @@
         <x:v>specs</x:v>
       </x:c>
       <x:c r="E28" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:81</x:v>
+        <x:v>src/语法分析/parser.cpp:71</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
@@ -811,7 +811,7 @@
         <x:v>specs</x:v>
       </x:c>
       <x:c r="E29" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:81</x:v>
+        <x:v>src/语法分析/parser.cpp:71</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
@@ -828,7 +828,7 @@
         <x:v>specs</x:v>
       </x:c>
       <x:c r="E30" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:81</x:v>
+        <x:v>src/语法分析/parser.cpp:71</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
@@ -845,7 +845,7 @@
         <x:v>specs</x:v>
       </x:c>
       <x:c r="E31" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:81</x:v>
+        <x:v>src/语法分析/parser.cpp:71</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
@@ -862,7 +862,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E32" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
@@ -879,7 +879,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E33" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="24" customHeight="1">
@@ -896,7 +896,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E34" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
@@ -913,7 +913,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E35" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="24" customHeight="1">
@@ -930,7 +930,7 @@
         <x:v>declaration</x:v>
       </x:c>
       <x:c r="E36" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:122</x:v>
+        <x:v>src/语法分析/parser.cpp:112</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="24" customHeight="1">
@@ -947,7 +947,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E37" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:93</x:v>
+        <x:v>src/语法分析/parser.cpp:83</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="24" customHeight="1">
@@ -964,7 +964,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E38" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:93</x:v>
+        <x:v>src/语法分析/parser.cpp:83</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="24" customHeight="1">
@@ -981,7 +981,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E39" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:93</x:v>
+        <x:v>src/语法分析/parser.cpp:83</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="24" customHeight="1">
@@ -998,7 +998,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E40" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:93</x:v>
+        <x:v>src/语法分析/parser.cpp:83</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="24" customHeight="1">
@@ -1015,7 +1015,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E41" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:93</x:v>
+        <x:v>src/语法分析/parser.cpp:83</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="24" customHeight="1">
@@ -1032,7 +1032,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E42" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:93</x:v>
+        <x:v>src/语法分析/parser.cpp:83</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="24" customHeight="1">
@@ -1049,7 +1049,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E43" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:93</x:v>
+        <x:v>src/语法分析/parser.cpp:83</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="24" customHeight="1">
@@ -1066,7 +1066,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E44" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:93</x:v>
+        <x:v>src/语法分析/parser.cpp:83</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="24" customHeight="1">
@@ -1083,7 +1083,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E45" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:93</x:v>
+        <x:v>src/语法分析/parser.cpp:83</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="24" customHeight="1">
@@ -1100,7 +1100,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E46" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:93</x:v>
+        <x:v>src/语法分析/parser.cpp:83</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="24" customHeight="1">
@@ -1117,7 +1117,7 @@
         <x:v>declarator</x:v>
       </x:c>
       <x:c r="E47" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:93</x:v>
+        <x:v>src/语法分析/parser.cpp:83</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="24" customHeight="1">
@@ -1134,7 +1134,7 @@
         <x:v>block</x:v>
       </x:c>
       <x:c r="E48" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:147</x:v>
+        <x:v>src/语法分析/parser.cpp:137</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="24" customHeight="1">
@@ -1151,7 +1151,7 @@
         <x:v>block</x:v>
       </x:c>
       <x:c r="E49" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:147</x:v>
+        <x:v>src/语法分析/parser.cpp:137</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="24" customHeight="1">
@@ -1168,7 +1168,7 @@
         <x:v>block</x:v>
       </x:c>
       <x:c r="E50" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:147</x:v>
+        <x:v>src/语法分析/parser.cpp:137</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="24" customHeight="1">
@@ -1185,7 +1185,7 @@
         <x:v>block</x:v>
       </x:c>
       <x:c r="E51" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:147</x:v>
+        <x:v>src/语法分析/parser.cpp:137</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="24" customHeight="1">
@@ -1202,7 +1202,7 @@
         <x:v>block</x:v>
       </x:c>
       <x:c r="E52" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:147</x:v>
+        <x:v>src/语法分析/parser.cpp:137</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="24" customHeight="1">
@@ -1219,7 +1219,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E53" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:153</x:v>
+        <x:v>src/语法分析/parser.cpp:143</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="24" customHeight="1">
@@ -1236,7 +1236,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E54" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:153</x:v>
+        <x:v>src/语法分析/parser.cpp:143</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="24" customHeight="1">
@@ -1253,7 +1253,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E55" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:153</x:v>
+        <x:v>src/语法分析/parser.cpp:143</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="24" customHeight="1">
@@ -1270,7 +1270,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E56" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:153</x:v>
+        <x:v>src/语法分析/parser.cpp:143</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="24" customHeight="1">
@@ -1287,7 +1287,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E57" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:153</x:v>
+        <x:v>src/语法分析/parser.cpp:143</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="24" customHeight="1">
@@ -1304,7 +1304,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E58" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:153</x:v>
+        <x:v>src/语法分析/parser.cpp:143</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="24" customHeight="1">
@@ -1321,7 +1321,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E59" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:153</x:v>
+        <x:v>src/语法分析/parser.cpp:143</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="24" customHeight="1">
@@ -1338,7 +1338,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E60" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:153</x:v>
+        <x:v>src/语法分析/parser.cpp:143</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="24" customHeight="1">
@@ -1355,7 +1355,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E61" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:153</x:v>
+        <x:v>src/语法分析/parser.cpp:143</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="24" customHeight="1">
@@ -1372,7 +1372,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E62" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:153</x:v>
+        <x:v>src/语法分析/parser.cpp:143</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="24" customHeight="1">
@@ -1389,7 +1389,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E63" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:153</x:v>
+        <x:v>src/语法分析/parser.cpp:143</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="24" customHeight="1">
@@ -1406,7 +1406,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E64" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:153</x:v>
+        <x:v>src/语法分析/parser.cpp:143</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="24" customHeight="1">
@@ -1423,7 +1423,7 @@
         <x:v>statement</x:v>
       </x:c>
       <x:c r="E65" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:153</x:v>
+        <x:v>src/语法分析/parser.cpp:143</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="24" customHeight="1">
@@ -1440,7 +1440,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E66" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="24" customHeight="1">
@@ -1457,7 +1457,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E67" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="24" customHeight="1">
@@ -1474,7 +1474,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E68" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="24" customHeight="1">
@@ -1491,7 +1491,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E69" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="24" customHeight="1">
@@ -1508,7 +1508,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E70" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="24" customHeight="1">
@@ -1525,7 +1525,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E71" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="24" customHeight="1">
@@ -1542,7 +1542,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E72" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="24" customHeight="1">
@@ -1559,7 +1559,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E73" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="24" customHeight="1">
@@ -1576,7 +1576,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E74" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="24" customHeight="1">
@@ -1593,7 +1593,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E75" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="24" customHeight="1">
@@ -1610,7 +1610,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E76" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="24" customHeight="1">
@@ -1627,7 +1627,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E77" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="24" customHeight="1">
@@ -1644,7 +1644,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E78" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="24" customHeight="1">
@@ -1661,7 +1661,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E79" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="24" customHeight="1">
@@ -1678,7 +1678,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E80" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="24" customHeight="1">
@@ -1695,7 +1695,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E81" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="24" customHeight="1">
@@ -1712,7 +1712,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E82" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="24" customHeight="1">
@@ -1729,7 +1729,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E83" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="24" customHeight="1">
@@ -1746,7 +1746,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E84" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="24" customHeight="1">
@@ -1763,7 +1763,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E85" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="24" customHeight="1">
@@ -1780,7 +1780,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E86" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="24" customHeight="1">
@@ -1797,7 +1797,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E87" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="24" customHeight="1">
@@ -1814,7 +1814,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E88" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="24" customHeight="1">
@@ -1831,7 +1831,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E89" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="24" customHeight="1">
@@ -1848,7 +1848,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E90" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="24" customHeight="1">
@@ -1865,7 +1865,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E91" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="24" customHeight="1">
@@ -1882,7 +1882,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E92" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="24" customHeight="1">
@@ -1899,7 +1899,7 @@
         <x:v>expression</x:v>
       </x:c>
       <x:c r="E93" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:179</x:v>
+        <x:v>src/语法分析/parser.cpp:169</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="24" customHeight="1">
@@ -1916,7 +1916,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E94" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="24" customHeight="1">
@@ -1933,7 +1933,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E95" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="24" customHeight="1">
@@ -1950,7 +1950,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E96" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="24" customHeight="1">
@@ -1967,7 +1967,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E97" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="24" customHeight="1">
@@ -1984,7 +1984,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E98" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="24" customHeight="1">
@@ -2001,7 +2001,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E99" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="24" customHeight="1">
@@ -2018,7 +2018,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E100" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="24" customHeight="1">
@@ -2035,7 +2035,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E101" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="24" customHeight="1">
@@ -2052,7 +2052,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E102" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="24" customHeight="1">
@@ -2069,7 +2069,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E103" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="24" customHeight="1">
@@ -2086,7 +2086,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E104" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="24" customHeight="1">
@@ -2103,7 +2103,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E105" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="24" customHeight="1">
@@ -2120,7 +2120,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E106" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="24" customHeight="1">
@@ -2137,7 +2137,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E107" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="24" customHeight="1">
@@ -2154,7 +2154,7 @@
         <x:v>unary</x:v>
       </x:c>
       <x:c r="E108" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:190</x:v>
+        <x:v>src/语法分析/parser.cpp:180</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="24" customHeight="1">
@@ -2171,7 +2171,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E109" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:217</x:v>
+        <x:v>src/语法分析/parser.cpp:207</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="24" customHeight="1">
@@ -2188,7 +2188,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E110" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:217</x:v>
+        <x:v>src/语法分析/parser.cpp:207</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="24" customHeight="1">
@@ -2205,7 +2205,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E111" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:217</x:v>
+        <x:v>src/语法分析/parser.cpp:207</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="24" customHeight="1">
@@ -2222,7 +2222,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E112" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:217</x:v>
+        <x:v>src/语法分析/parser.cpp:207</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="24" customHeight="1">
@@ -2239,7 +2239,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E113" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:217</x:v>
+        <x:v>src/语法分析/parser.cpp:207</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="24" customHeight="1">
@@ -2256,7 +2256,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E114" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:217</x:v>
+        <x:v>src/语法分析/parser.cpp:207</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="24" customHeight="1">
@@ -2273,7 +2273,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E115" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:217</x:v>
+        <x:v>src/语法分析/parser.cpp:207</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="24" customHeight="1">
@@ -2290,7 +2290,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E116" s="17" t="str">
-        <x:v>src/语法分析/parser.cpp:217</x:v>
+        <x:v>src/语法分析/parser.cpp:207</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="24" customHeight="1">
@@ -2307,7 +2307,7 @@
         <x:v>postfix</x:v>
       </x:c>
       <x:c r="E117" s="18" t="str">
-        <x:v>src/语法分析/parser.cpp:217</x:v>
+        <x:v>src/语法分析/parser.cpp:207</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2318,7 +2318,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde842d4fbcc04a0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbcdc065839e4d46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>